<commit_message>
Updating BC, Gantt, Master Usecase
BC: Update costs due to Mortens withdrawal
Gantt: Update actual starts and progress
Master Usecase: Update requirements
</commit_message>
<xml_diff>
--- a/PROJECT/Gantt project planner.xlsx
+++ b/PROJECT/Gantt project planner.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B4772C7-E8F5-45B9-8FC1-78F7C4677A97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C910C2B-8FDA-4E79-8803-30A89FB92E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
   <si>
     <t>Project Planner</t>
   </si>
@@ -181,15 +181,9 @@
     <t>Setting up</t>
   </si>
   <si>
-    <t>Programming</t>
-  </si>
-  <si>
     <t>Testing:</t>
   </si>
   <si>
-    <t>Setting up Enviorment</t>
-  </si>
-  <si>
     <t>Cyclic Tests</t>
   </si>
   <si>
@@ -211,13 +205,16 @@
     <t>Design</t>
   </si>
   <si>
-    <t>Analyse</t>
-  </si>
-  <si>
     <t>Coding</t>
   </si>
   <si>
-    <t>Analyse:</t>
+    <t>Analysis</t>
+  </si>
+  <si>
+    <t>Analysis:</t>
+  </si>
+  <si>
+    <t>Implementing</t>
   </si>
 </sst>
 </file>
@@ -1401,7 +1398,7 @@
     </row>
     <row r="6" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="24" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C6" s="19">
         <v>1</v>
@@ -1421,13 +1418,13 @@
     </row>
     <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="24" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C7" s="19">
         <v>7</v>
       </c>
       <c r="D7" s="19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E7" s="19">
         <v>9</v>
@@ -1435,7 +1432,9 @@
       <c r="F7" s="21">
         <v>3</v>
       </c>
-      <c r="G7" s="23"/>
+      <c r="G7" s="23">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="24" t="s">
@@ -1450,32 +1449,40 @@
       <c r="E8" s="19">
         <v>13</v>
       </c>
-      <c r="F8" s="21"/>
-      <c r="G8" s="23"/>
+      <c r="F8" s="21">
+        <v>18</v>
+      </c>
+      <c r="G8" s="23">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="9" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="24" t="s">
         <v>16</v>
       </c>
       <c r="C9" s="19">
+        <v>20</v>
+      </c>
+      <c r="D9" s="19">
         <v>13</v>
       </c>
-      <c r="D9" s="19">
-        <v>10</v>
-      </c>
-      <c r="E9" s="19"/>
+      <c r="E9" s="19">
+        <v>19</v>
+      </c>
       <c r="F9" s="21"/>
-      <c r="G9" s="23"/>
+      <c r="G9" s="23">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
       <c r="C10" s="19">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D10" s="19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" s="19"/>
       <c r="F10" s="21"/>
@@ -1486,7 +1493,7 @@
         <v>18</v>
       </c>
       <c r="C11" s="19">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D11" s="19">
         <v>1</v>
@@ -1505,7 +1512,7 @@
     </row>
     <row r="13" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="26" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C13" s="19"/>
       <c r="D13" s="19"/>
@@ -1529,7 +1536,9 @@
       <c r="F14" s="21">
         <v>4</v>
       </c>
-      <c r="G14" s="23"/>
+      <c r="G14" s="23">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="24" t="s">
@@ -1547,25 +1556,29 @@
       <c r="F15" s="21">
         <v>4</v>
       </c>
-      <c r="G15" s="23"/>
+      <c r="G15" s="23">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="24" t="s">
         <v>21</v>
       </c>
       <c r="C16" s="20">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D16" s="19">
         <v>1</v>
       </c>
       <c r="E16" s="19">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F16" s="21">
-        <v>1</v>
-      </c>
-      <c r="G16" s="23"/>
+        <v>2</v>
+      </c>
+      <c r="G16" s="23">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="24" t="s">
@@ -1583,7 +1596,9 @@
       <c r="F17" s="21">
         <v>4</v>
       </c>
-      <c r="G17" s="23"/>
+      <c r="G17" s="23">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="18"/>
@@ -1608,32 +1623,38 @@
         <v>24</v>
       </c>
       <c r="C20" s="19">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D20" s="19">
         <v>5</v>
       </c>
       <c r="E20" s="19">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F20" s="21">
         <v>3</v>
       </c>
-      <c r="G20" s="23"/>
+      <c r="G20" s="23">
+        <v>1</v>
+      </c>
     </row>
     <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="24" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C21" s="19">
-        <v>13</v>
-      </c>
-      <c r="D21" s="19"/>
+        <v>18</v>
+      </c>
+      <c r="D21" s="19">
+        <v>15</v>
+      </c>
       <c r="E21" s="19">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F21" s="21"/>
-      <c r="G21" s="23"/>
+      <c r="G21" s="23">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="18"/>
@@ -1645,7 +1666,7 @@
     </row>
     <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="26" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C23" s="19"/>
       <c r="D23" s="19"/>
@@ -1655,20 +1676,34 @@
     </row>
     <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="21"/>
-      <c r="G24" s="23"/>
+        <v>24</v>
+      </c>
+      <c r="C24" s="19">
+        <v>20</v>
+      </c>
+      <c r="D24" s="19">
+        <v>3</v>
+      </c>
+      <c r="E24" s="19">
+        <v>19</v>
+      </c>
+      <c r="F24" s="21">
+        <v>4</v>
+      </c>
+      <c r="G24" s="23">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
+        <v>26</v>
+      </c>
+      <c r="C25" s="19">
+        <v>23</v>
+      </c>
+      <c r="D25" s="19">
+        <v>10</v>
+      </c>
       <c r="E25" s="19"/>
       <c r="F25" s="21"/>
       <c r="G25" s="23"/>
@@ -1683,7 +1718,7 @@
     </row>
     <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="26" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C27" s="19"/>
       <c r="D27" s="19"/>
@@ -1693,20 +1728,28 @@
     </row>
     <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
+        <v>28</v>
+      </c>
+      <c r="C28" s="19">
+        <v>33</v>
+      </c>
+      <c r="D28" s="19">
+        <v>1</v>
+      </c>
       <c r="E28" s="19"/>
       <c r="F28" s="21"/>
       <c r="G28" s="23"/>
     </row>
     <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
+        <v>29</v>
+      </c>
+      <c r="C29" s="19">
+        <v>34</v>
+      </c>
+      <c r="D29" s="19">
+        <v>1</v>
+      </c>
       <c r="E29" s="19"/>
       <c r="F29" s="21"/>
       <c r="G29" s="23"/>
@@ -1721,7 +1764,7 @@
     </row>
     <row r="31" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B31" s="26" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C31" s="19"/>
       <c r="D31" s="19"/>
@@ -1731,10 +1774,14 @@
     </row>
     <row r="32" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
+        <v>31</v>
+      </c>
+      <c r="C32" s="19">
+        <v>34</v>
+      </c>
+      <c r="D32" s="19">
+        <v>1</v>
+      </c>
       <c r="E32" s="19"/>
       <c r="F32" s="21"/>
       <c r="G32" s="23"/>

</xml_diff>

<commit_message>
Update Gantt project planner.xlsx
</commit_message>
<xml_diff>
--- a/PROJECT/Gantt project planner.xlsx
+++ b/PROJECT/Gantt project planner.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C910C2B-8FDA-4E79-8803-30A89FB92E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19A47853-ACC7-44D9-A279-EF4F54167480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Planner" sheetId="1" r:id="rId1"/>
@@ -1078,17 +1078,17 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:BO35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="2.77734375" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="2.75" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.6640625" customWidth="1"/>
-    <col min="2" max="2" width="22.88671875" style="2" customWidth="1"/>
-    <col min="3" max="6" width="11.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.6640625" style="4" customWidth="1"/>
-    <col min="8" max="27" width="2.77734375" style="1"/>
-    <col min="33" max="33" width="2.77734375" customWidth="1"/>
+    <col min="1" max="1" width="2.625" customWidth="1"/>
+    <col min="2" max="2" width="22.875" style="2" customWidth="1"/>
+    <col min="3" max="6" width="11.625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.625" style="4" customWidth="1"/>
+    <col min="8" max="27" width="2.75" style="1"/>
+    <col min="33" max="33" width="2.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:67" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="1.05">
+    <row r="1" spans="2:67" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.85">
       <c r="B1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1098,7 +1098,7 @@
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
     </row>
-    <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="17" t="s">
         <v>14</v>
       </c>
@@ -1156,7 +1156,7 @@
       <c r="AO2" s="28"/>
       <c r="AP2" s="28"/>
     </row>
-    <row r="3" spans="2:67" s="7" customFormat="1" ht="39.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:67" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B3" s="29" t="s">
         <v>2</v>
       </c>
@@ -1198,7 +1198,7 @@
       <c r="Z3" s="6"/>
       <c r="AA3" s="6"/>
     </row>
-    <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="30"/>
       <c r="C4" s="32"/>
       <c r="D4" s="32"/>
@@ -1386,7 +1386,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="26" t="s">
         <v>15</v>
       </c>
@@ -1396,7 +1396,7 @@
       <c r="F5" s="21"/>
       <c r="G5" s="23"/>
     </row>
-    <row r="6" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="24" t="s">
         <v>34</v>
       </c>
@@ -1416,7 +1416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="24" t="s">
         <v>32</v>
       </c>
@@ -1436,7 +1436,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="24" t="s">
         <v>36</v>
       </c>
@@ -1453,10 +1453,10 @@
         <v>18</v>
       </c>
       <c r="G8" s="23">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="9" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="24" t="s">
         <v>16</v>
       </c>
@@ -1471,10 +1471,10 @@
       </c>
       <c r="F9" s="21"/>
       <c r="G9" s="23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
@@ -1484,11 +1484,15 @@
       <c r="D10" s="19">
         <v>2</v>
       </c>
-      <c r="E10" s="19"/>
+      <c r="E10" s="19">
+        <v>31</v>
+      </c>
       <c r="F10" s="21"/>
-      <c r="G10" s="23"/>
-    </row>
-    <row r="11" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G10" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="11" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="24" t="s">
         <v>18</v>
       </c>
@@ -1502,7 +1506,7 @@
       <c r="F11" s="21"/>
       <c r="G11" s="23"/>
     </row>
-    <row r="12" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="18"/>
       <c r="C12" s="19"/>
       <c r="D12" s="19"/>
@@ -1510,7 +1514,7 @@
       <c r="F12" s="21"/>
       <c r="G12" s="23"/>
     </row>
-    <row r="13" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="26" t="s">
         <v>35</v>
       </c>
@@ -1520,7 +1524,7 @@
       <c r="F13" s="21"/>
       <c r="G13" s="23"/>
     </row>
-    <row r="14" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="24" t="s">
         <v>19</v>
       </c>
@@ -1540,7 +1544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="24" t="s">
         <v>20</v>
       </c>
@@ -1560,7 +1564,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="24" t="s">
         <v>21</v>
       </c>
@@ -1577,10 +1581,10 @@
         <v>2</v>
       </c>
       <c r="G16" s="23">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="24" t="s">
         <v>22</v>
       </c>
@@ -1600,7 +1604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="18"/>
       <c r="C18" s="19"/>
       <c r="D18" s="19"/>
@@ -1608,7 +1612,7 @@
       <c r="F18" s="21"/>
       <c r="G18" s="23"/>
     </row>
-    <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="26" t="s">
         <v>23</v>
       </c>
@@ -1618,7 +1622,7 @@
       <c r="F19" s="21"/>
       <c r="G19" s="23"/>
     </row>
-    <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="24" t="s">
         <v>24</v>
       </c>
@@ -1638,7 +1642,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="24" t="s">
         <v>33</v>
       </c>
@@ -1653,10 +1657,10 @@
       </c>
       <c r="F21" s="21"/>
       <c r="G21" s="23">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="18"/>
       <c r="C22" s="19"/>
       <c r="D22" s="19"/>
@@ -1664,7 +1668,7 @@
       <c r="F22" s="21"/>
       <c r="G22" s="23"/>
     </row>
-    <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="26" t="s">
         <v>25</v>
       </c>
@@ -1674,7 +1678,7 @@
       <c r="F23" s="21"/>
       <c r="G23" s="23"/>
     </row>
-    <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="24" t="s">
         <v>24</v>
       </c>
@@ -1691,10 +1695,10 @@
         <v>4</v>
       </c>
       <c r="G24" s="23">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="24" t="s">
         <v>26</v>
       </c>
@@ -1704,11 +1708,15 @@
       <c r="D25" s="19">
         <v>10</v>
       </c>
-      <c r="E25" s="19"/>
+      <c r="E25" s="19">
+        <v>23</v>
+      </c>
       <c r="F25" s="21"/>
-      <c r="G25" s="23"/>
-    </row>
-    <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G25" s="23">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="18"/>
       <c r="C26" s="19"/>
       <c r="D26" s="19"/>
@@ -1716,7 +1724,7 @@
       <c r="F26" s="21"/>
       <c r="G26" s="23"/>
     </row>
-    <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="26" t="s">
         <v>27</v>
       </c>
@@ -1726,7 +1734,7 @@
       <c r="F27" s="21"/>
       <c r="G27" s="23"/>
     </row>
-    <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="24" t="s">
         <v>28</v>
       </c>
@@ -1736,11 +1744,15 @@
       <c r="D28" s="19">
         <v>1</v>
       </c>
-      <c r="E28" s="19"/>
+      <c r="E28" s="19">
+        <v>31</v>
+      </c>
       <c r="F28" s="21"/>
-      <c r="G28" s="23"/>
-    </row>
-    <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G28" s="23">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="24" t="s">
         <v>29</v>
       </c>
@@ -1754,7 +1766,7 @@
       <c r="F29" s="21"/>
       <c r="G29" s="23"/>
     </row>
-    <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="18"/>
       <c r="C30" s="19"/>
       <c r="D30" s="19"/>
@@ -1762,7 +1774,7 @@
       <c r="F30" s="21"/>
       <c r="G30" s="23"/>
     </row>
-    <row r="31" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="26" t="s">
         <v>30</v>
       </c>
@@ -1772,7 +1784,7 @@
       <c r="F31" s="21"/>
       <c r="G31" s="23"/>
     </row>
-    <row r="32" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="24" t="s">
         <v>31</v>
       </c>
@@ -1786,7 +1798,7 @@
       <c r="F32" s="21"/>
       <c r="G32" s="23"/>
     </row>
-    <row r="33" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="18"/>
       <c r="C33" s="19"/>
       <c r="D33" s="19"/>
@@ -1794,7 +1806,7 @@
       <c r="F33" s="21"/>
       <c r="G33" s="23"/>
     </row>
-    <row r="34" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="18"/>
       <c r="C34" s="19"/>
       <c r="D34" s="19"/>
@@ -1802,7 +1814,7 @@
       <c r="F34" s="21"/>
       <c r="G34" s="23"/>
     </row>
-    <row r="35" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="18"/>
       <c r="C35" s="19"/>
       <c r="D35" s="19"/>

</xml_diff>

<commit_message>
Gantt complete,  MeetingMinutes complete
</commit_message>
<xml_diff>
--- a/PROJECT/Gantt project planner.xlsx
+++ b/PROJECT/Gantt project planner.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19A47853-ACC7-44D9-A279-EF4F54167480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{881200D9-CBFC-44CF-BE49-B8D6BD414B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Planner" sheetId="1" r:id="rId1"/>
@@ -1078,17 +1078,17 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:BO35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="2.75" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="2.77734375" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.625" customWidth="1"/>
-    <col min="2" max="2" width="22.875" style="2" customWidth="1"/>
-    <col min="3" max="6" width="11.625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.625" style="4" customWidth="1"/>
-    <col min="8" max="27" width="2.75" style="1"/>
-    <col min="33" max="33" width="2.75" customWidth="1"/>
+    <col min="1" max="1" width="2.6640625" customWidth="1"/>
+    <col min="2" max="2" width="22.88671875" style="2" customWidth="1"/>
+    <col min="3" max="6" width="11.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" style="4" customWidth="1"/>
+    <col min="8" max="27" width="2.77734375" style="1"/>
+    <col min="33" max="33" width="2.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:67" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:67" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="1.05">
       <c r="B1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1098,7 +1098,7 @@
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
     </row>
-    <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="17" t="s">
         <v>14</v>
       </c>
@@ -1156,7 +1156,7 @@
       <c r="AO2" s="28"/>
       <c r="AP2" s="28"/>
     </row>
-    <row r="3" spans="2:67" s="7" customFormat="1" ht="39.950000000000003" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:67" s="7" customFormat="1" ht="39.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B3" s="29" t="s">
         <v>2</v>
       </c>
@@ -1198,7 +1198,7 @@
       <c r="Z3" s="6"/>
       <c r="AA3" s="6"/>
     </row>
-    <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="30"/>
       <c r="C4" s="32"/>
       <c r="D4" s="32"/>
@@ -1386,7 +1386,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="26" t="s">
         <v>15</v>
       </c>
@@ -1396,7 +1396,7 @@
       <c r="F5" s="21"/>
       <c r="G5" s="23"/>
     </row>
-    <row r="6" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="24" t="s">
         <v>34</v>
       </c>
@@ -1416,7 +1416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="24" t="s">
         <v>32</v>
       </c>
@@ -1436,7 +1436,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="24" t="s">
         <v>36</v>
       </c>
@@ -1456,7 +1456,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="24" t="s">
         <v>16</v>
       </c>
@@ -1469,12 +1469,14 @@
       <c r="E9" s="19">
         <v>19</v>
       </c>
-      <c r="F9" s="21"/>
+      <c r="F9" s="21">
+        <v>13</v>
+      </c>
       <c r="G9" s="23">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="24" t="s">
         <v>17</v>
       </c>
@@ -1487,12 +1489,14 @@
       <c r="E10" s="19">
         <v>31</v>
       </c>
-      <c r="F10" s="21"/>
+      <c r="F10" s="21">
+        <v>2</v>
+      </c>
       <c r="G10" s="23">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="11" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="24" t="s">
         <v>18</v>
       </c>
@@ -1502,11 +1506,17 @@
       <c r="D11" s="19">
         <v>1</v>
       </c>
-      <c r="E11" s="19"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="23"/>
-    </row>
-    <row r="12" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E11" s="19">
+        <v>34</v>
+      </c>
+      <c r="F11" s="21">
+        <v>1</v>
+      </c>
+      <c r="G11" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="18"/>
       <c r="C12" s="19"/>
       <c r="D12" s="19"/>
@@ -1514,7 +1524,7 @@
       <c r="F12" s="21"/>
       <c r="G12" s="23"/>
     </row>
-    <row r="13" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="26" t="s">
         <v>35</v>
       </c>
@@ -1524,7 +1534,7 @@
       <c r="F13" s="21"/>
       <c r="G13" s="23"/>
     </row>
-    <row r="14" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="24" t="s">
         <v>19</v>
       </c>
@@ -1544,7 +1554,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="24" t="s">
         <v>20</v>
       </c>
@@ -1564,7 +1574,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="24" t="s">
         <v>21</v>
       </c>
@@ -1584,7 +1594,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="24" t="s">
         <v>22</v>
       </c>
@@ -1604,7 +1614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="18"/>
       <c r="C18" s="19"/>
       <c r="D18" s="19"/>
@@ -1612,7 +1622,7 @@
       <c r="F18" s="21"/>
       <c r="G18" s="23"/>
     </row>
-    <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="26" t="s">
         <v>23</v>
       </c>
@@ -1622,7 +1632,7 @@
       <c r="F19" s="21"/>
       <c r="G19" s="23"/>
     </row>
-    <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="24" t="s">
         <v>24</v>
       </c>
@@ -1642,7 +1652,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="24" t="s">
         <v>33</v>
       </c>
@@ -1660,7 +1670,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="18"/>
       <c r="C22" s="19"/>
       <c r="D22" s="19"/>
@@ -1668,7 +1678,7 @@
       <c r="F22" s="21"/>
       <c r="G22" s="23"/>
     </row>
-    <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="26" t="s">
         <v>25</v>
       </c>
@@ -1678,7 +1688,7 @@
       <c r="F23" s="21"/>
       <c r="G23" s="23"/>
     </row>
-    <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="24" t="s">
         <v>24</v>
       </c>
@@ -1698,7 +1708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="24" t="s">
         <v>26</v>
       </c>
@@ -1711,12 +1721,14 @@
       <c r="E25" s="19">
         <v>23</v>
       </c>
-      <c r="F25" s="21"/>
+      <c r="F25" s="21">
+        <v>9</v>
+      </c>
       <c r="G25" s="23">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="18"/>
       <c r="C26" s="19"/>
       <c r="D26" s="19"/>
@@ -1724,7 +1736,7 @@
       <c r="F26" s="21"/>
       <c r="G26" s="23"/>
     </row>
-    <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="26" t="s">
         <v>27</v>
       </c>
@@ -1734,7 +1746,7 @@
       <c r="F27" s="21"/>
       <c r="G27" s="23"/>
     </row>
-    <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="24" t="s">
         <v>28</v>
       </c>
@@ -1747,12 +1759,14 @@
       <c r="E28" s="19">
         <v>31</v>
       </c>
-      <c r="F28" s="21"/>
+      <c r="F28" s="21">
+        <v>2</v>
+      </c>
       <c r="G28" s="23">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="24" t="s">
         <v>29</v>
       </c>
@@ -1762,11 +1776,17 @@
       <c r="D29" s="19">
         <v>1</v>
       </c>
-      <c r="E29" s="19"/>
-      <c r="F29" s="21"/>
-      <c r="G29" s="23"/>
-    </row>
-    <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E29" s="19">
+        <v>34</v>
+      </c>
+      <c r="F29" s="21">
+        <v>1</v>
+      </c>
+      <c r="G29" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="18"/>
       <c r="C30" s="19"/>
       <c r="D30" s="19"/>
@@ -1774,7 +1794,7 @@
       <c r="F30" s="21"/>
       <c r="G30" s="23"/>
     </row>
-    <row r="31" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B31" s="26" t="s">
         <v>30</v>
       </c>
@@ -1784,7 +1804,7 @@
       <c r="F31" s="21"/>
       <c r="G31" s="23"/>
     </row>
-    <row r="32" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="24" t="s">
         <v>31</v>
       </c>
@@ -1794,11 +1814,17 @@
       <c r="D32" s="19">
         <v>1</v>
       </c>
-      <c r="E32" s="19"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="23"/>
-    </row>
-    <row r="33" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E32" s="19">
+        <v>34</v>
+      </c>
+      <c r="F32" s="21">
+        <v>1</v>
+      </c>
+      <c r="G32" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B33" s="18"/>
       <c r="C33" s="19"/>
       <c r="D33" s="19"/>
@@ -1806,7 +1832,7 @@
       <c r="F33" s="21"/>
       <c r="G33" s="23"/>
     </row>
-    <row r="34" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B34" s="18"/>
       <c r="C34" s="19"/>
       <c r="D34" s="19"/>
@@ -1814,7 +1840,7 @@
       <c r="F34" s="21"/>
       <c r="G34" s="23"/>
     </row>
-    <row r="35" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="18"/>
       <c r="C35" s="19"/>
       <c r="D35" s="19"/>

</xml_diff>